<commit_message>
Smart Revision part 1: spaced reviews, weak topics, Before-Exam Mode, bookmarks
- Migration: revision_states, append-only revision_reviews, exam_dates,
  revision_exam_modes, question_bookmarks, with RLS and cross-tenant tests
- Practice feeds the spaced-review schedule (1/3/7/14/30/60 days) per sub-topic
- Centre exam dates from a new Exams sheet in the timetable spreadsheet;
  students can add their own school exams
- Revision Home, Weak Topics, Before-Exam Mode, Bookmark Review, Materials (empty)
- Bookmark toggle in the practice runner
- ADR 0009, runbook and CLAUDE.md status

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EdB7jr7dZB3nArHF8Gftsp
</commit_message>
<xml_diff>
--- a/docs/templates/timetable-example-test-centre.xlsx
+++ b/docs/templates/timetable-example-test-centre.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="One-off sessions" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancellations" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exams" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -450,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -638,19 +639,36 @@
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
+          <t>Exams</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Exam dates for everyone on a course, e.g. P6 | Mathematics | PSLE | 26/9/2027. Students see them in Smart Revision → Before-Exam Mode. Listing a course's exams replaces its upcoming exams; leave the sheet empty to keep them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
           <t>Example (Classes)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>P5MA-SAT-0900 | P5 | Mathematics | Physical tutorial | Bishan | Room 1 | Ms Lim | Sat | 09:00 | 120 | 3/1/2027 | 30/12/2027 | 12 |</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>P6SC-WED-LIVE | P6 | Science | Live tutorial | | | Mr Ong | Wed | 19:30 | 90 | 6/1/2027 | 29/12/2027 | | https://zoom.us/j/123456789</t>
         </is>
@@ -10678,4 +10696,1563 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D501"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="D2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="D3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="D4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="D5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="D6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="D7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="D8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="D9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="D10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="D11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="D12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="D13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="D14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="D15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="D16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="D17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="D18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="D19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="D20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="D21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="D22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="D23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="D24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="D25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="D26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="D27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="D28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="D29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="D30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="D31" s="7" t="n"/>
+    </row>
+    <row r="32">
+      <c r="D32" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="D33" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="D34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="D35" s="7" t="n"/>
+    </row>
+    <row r="36">
+      <c r="D36" s="7" t="n"/>
+    </row>
+    <row r="37">
+      <c r="D37" s="7" t="n"/>
+    </row>
+    <row r="38">
+      <c r="D38" s="7" t="n"/>
+    </row>
+    <row r="39">
+      <c r="D39" s="7" t="n"/>
+    </row>
+    <row r="40">
+      <c r="D40" s="7" t="n"/>
+    </row>
+    <row r="41">
+      <c r="D41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="D42" s="7" t="n"/>
+    </row>
+    <row r="43">
+      <c r="D43" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="D44" s="7" t="n"/>
+    </row>
+    <row r="45">
+      <c r="D45" s="7" t="n"/>
+    </row>
+    <row r="46">
+      <c r="D46" s="7" t="n"/>
+    </row>
+    <row r="47">
+      <c r="D47" s="7" t="n"/>
+    </row>
+    <row r="48">
+      <c r="D48" s="7" t="n"/>
+    </row>
+    <row r="49">
+      <c r="D49" s="7" t="n"/>
+    </row>
+    <row r="50">
+      <c r="D50" s="7" t="n"/>
+    </row>
+    <row r="51">
+      <c r="D51" s="7" t="n"/>
+    </row>
+    <row r="52">
+      <c r="D52" s="7" t="n"/>
+    </row>
+    <row r="53">
+      <c r="D53" s="7" t="n"/>
+    </row>
+    <row r="54">
+      <c r="D54" s="7" t="n"/>
+    </row>
+    <row r="55">
+      <c r="D55" s="7" t="n"/>
+    </row>
+    <row r="56">
+      <c r="D56" s="7" t="n"/>
+    </row>
+    <row r="57">
+      <c r="D57" s="7" t="n"/>
+    </row>
+    <row r="58">
+      <c r="D58" s="7" t="n"/>
+    </row>
+    <row r="59">
+      <c r="D59" s="7" t="n"/>
+    </row>
+    <row r="60">
+      <c r="D60" s="7" t="n"/>
+    </row>
+    <row r="61">
+      <c r="D61" s="7" t="n"/>
+    </row>
+    <row r="62">
+      <c r="D62" s="7" t="n"/>
+    </row>
+    <row r="63">
+      <c r="D63" s="7" t="n"/>
+    </row>
+    <row r="64">
+      <c r="D64" s="7" t="n"/>
+    </row>
+    <row r="65">
+      <c r="D65" s="7" t="n"/>
+    </row>
+    <row r="66">
+      <c r="D66" s="7" t="n"/>
+    </row>
+    <row r="67">
+      <c r="D67" s="7" t="n"/>
+    </row>
+    <row r="68">
+      <c r="D68" s="7" t="n"/>
+    </row>
+    <row r="69">
+      <c r="D69" s="7" t="n"/>
+    </row>
+    <row r="70">
+      <c r="D70" s="7" t="n"/>
+    </row>
+    <row r="71">
+      <c r="D71" s="7" t="n"/>
+    </row>
+    <row r="72">
+      <c r="D72" s="7" t="n"/>
+    </row>
+    <row r="73">
+      <c r="D73" s="7" t="n"/>
+    </row>
+    <row r="74">
+      <c r="D74" s="7" t="n"/>
+    </row>
+    <row r="75">
+      <c r="D75" s="7" t="n"/>
+    </row>
+    <row r="76">
+      <c r="D76" s="7" t="n"/>
+    </row>
+    <row r="77">
+      <c r="D77" s="7" t="n"/>
+    </row>
+    <row r="78">
+      <c r="D78" s="7" t="n"/>
+    </row>
+    <row r="79">
+      <c r="D79" s="7" t="n"/>
+    </row>
+    <row r="80">
+      <c r="D80" s="7" t="n"/>
+    </row>
+    <row r="81">
+      <c r="D81" s="7" t="n"/>
+    </row>
+    <row r="82">
+      <c r="D82" s="7" t="n"/>
+    </row>
+    <row r="83">
+      <c r="D83" s="7" t="n"/>
+    </row>
+    <row r="84">
+      <c r="D84" s="7" t="n"/>
+    </row>
+    <row r="85">
+      <c r="D85" s="7" t="n"/>
+    </row>
+    <row r="86">
+      <c r="D86" s="7" t="n"/>
+    </row>
+    <row r="87">
+      <c r="D87" s="7" t="n"/>
+    </row>
+    <row r="88">
+      <c r="D88" s="7" t="n"/>
+    </row>
+    <row r="89">
+      <c r="D89" s="7" t="n"/>
+    </row>
+    <row r="90">
+      <c r="D90" s="7" t="n"/>
+    </row>
+    <row r="91">
+      <c r="D91" s="7" t="n"/>
+    </row>
+    <row r="92">
+      <c r="D92" s="7" t="n"/>
+    </row>
+    <row r="93">
+      <c r="D93" s="7" t="n"/>
+    </row>
+    <row r="94">
+      <c r="D94" s="7" t="n"/>
+    </row>
+    <row r="95">
+      <c r="D95" s="7" t="n"/>
+    </row>
+    <row r="96">
+      <c r="D96" s="7" t="n"/>
+    </row>
+    <row r="97">
+      <c r="D97" s="7" t="n"/>
+    </row>
+    <row r="98">
+      <c r="D98" s="7" t="n"/>
+    </row>
+    <row r="99">
+      <c r="D99" s="7" t="n"/>
+    </row>
+    <row r="100">
+      <c r="D100" s="7" t="n"/>
+    </row>
+    <row r="101">
+      <c r="D101" s="7" t="n"/>
+    </row>
+    <row r="102">
+      <c r="D102" s="7" t="n"/>
+    </row>
+    <row r="103">
+      <c r="D103" s="7" t="n"/>
+    </row>
+    <row r="104">
+      <c r="D104" s="7" t="n"/>
+    </row>
+    <row r="105">
+      <c r="D105" s="7" t="n"/>
+    </row>
+    <row r="106">
+      <c r="D106" s="7" t="n"/>
+    </row>
+    <row r="107">
+      <c r="D107" s="7" t="n"/>
+    </row>
+    <row r="108">
+      <c r="D108" s="7" t="n"/>
+    </row>
+    <row r="109">
+      <c r="D109" s="7" t="n"/>
+    </row>
+    <row r="110">
+      <c r="D110" s="7" t="n"/>
+    </row>
+    <row r="111">
+      <c r="D111" s="7" t="n"/>
+    </row>
+    <row r="112">
+      <c r="D112" s="7" t="n"/>
+    </row>
+    <row r="113">
+      <c r="D113" s="7" t="n"/>
+    </row>
+    <row r="114">
+      <c r="D114" s="7" t="n"/>
+    </row>
+    <row r="115">
+      <c r="D115" s="7" t="n"/>
+    </row>
+    <row r="116">
+      <c r="D116" s="7" t="n"/>
+    </row>
+    <row r="117">
+      <c r="D117" s="7" t="n"/>
+    </row>
+    <row r="118">
+      <c r="D118" s="7" t="n"/>
+    </row>
+    <row r="119">
+      <c r="D119" s="7" t="n"/>
+    </row>
+    <row r="120">
+      <c r="D120" s="7" t="n"/>
+    </row>
+    <row r="121">
+      <c r="D121" s="7" t="n"/>
+    </row>
+    <row r="122">
+      <c r="D122" s="7" t="n"/>
+    </row>
+    <row r="123">
+      <c r="D123" s="7" t="n"/>
+    </row>
+    <row r="124">
+      <c r="D124" s="7" t="n"/>
+    </row>
+    <row r="125">
+      <c r="D125" s="7" t="n"/>
+    </row>
+    <row r="126">
+      <c r="D126" s="7" t="n"/>
+    </row>
+    <row r="127">
+      <c r="D127" s="7" t="n"/>
+    </row>
+    <row r="128">
+      <c r="D128" s="7" t="n"/>
+    </row>
+    <row r="129">
+      <c r="D129" s="7" t="n"/>
+    </row>
+    <row r="130">
+      <c r="D130" s="7" t="n"/>
+    </row>
+    <row r="131">
+      <c r="D131" s="7" t="n"/>
+    </row>
+    <row r="132">
+      <c r="D132" s="7" t="n"/>
+    </row>
+    <row r="133">
+      <c r="D133" s="7" t="n"/>
+    </row>
+    <row r="134">
+      <c r="D134" s="7" t="n"/>
+    </row>
+    <row r="135">
+      <c r="D135" s="7" t="n"/>
+    </row>
+    <row r="136">
+      <c r="D136" s="7" t="n"/>
+    </row>
+    <row r="137">
+      <c r="D137" s="7" t="n"/>
+    </row>
+    <row r="138">
+      <c r="D138" s="7" t="n"/>
+    </row>
+    <row r="139">
+      <c r="D139" s="7" t="n"/>
+    </row>
+    <row r="140">
+      <c r="D140" s="7" t="n"/>
+    </row>
+    <row r="141">
+      <c r="D141" s="7" t="n"/>
+    </row>
+    <row r="142">
+      <c r="D142" s="7" t="n"/>
+    </row>
+    <row r="143">
+      <c r="D143" s="7" t="n"/>
+    </row>
+    <row r="144">
+      <c r="D144" s="7" t="n"/>
+    </row>
+    <row r="145">
+      <c r="D145" s="7" t="n"/>
+    </row>
+    <row r="146">
+      <c r="D146" s="7" t="n"/>
+    </row>
+    <row r="147">
+      <c r="D147" s="7" t="n"/>
+    </row>
+    <row r="148">
+      <c r="D148" s="7" t="n"/>
+    </row>
+    <row r="149">
+      <c r="D149" s="7" t="n"/>
+    </row>
+    <row r="150">
+      <c r="D150" s="7" t="n"/>
+    </row>
+    <row r="151">
+      <c r="D151" s="7" t="n"/>
+    </row>
+    <row r="152">
+      <c r="D152" s="7" t="n"/>
+    </row>
+    <row r="153">
+      <c r="D153" s="7" t="n"/>
+    </row>
+    <row r="154">
+      <c r="D154" s="7" t="n"/>
+    </row>
+    <row r="155">
+      <c r="D155" s="7" t="n"/>
+    </row>
+    <row r="156">
+      <c r="D156" s="7" t="n"/>
+    </row>
+    <row r="157">
+      <c r="D157" s="7" t="n"/>
+    </row>
+    <row r="158">
+      <c r="D158" s="7" t="n"/>
+    </row>
+    <row r="159">
+      <c r="D159" s="7" t="n"/>
+    </row>
+    <row r="160">
+      <c r="D160" s="7" t="n"/>
+    </row>
+    <row r="161">
+      <c r="D161" s="7" t="n"/>
+    </row>
+    <row r="162">
+      <c r="D162" s="7" t="n"/>
+    </row>
+    <row r="163">
+      <c r="D163" s="7" t="n"/>
+    </row>
+    <row r="164">
+      <c r="D164" s="7" t="n"/>
+    </row>
+    <row r="165">
+      <c r="D165" s="7" t="n"/>
+    </row>
+    <row r="166">
+      <c r="D166" s="7" t="n"/>
+    </row>
+    <row r="167">
+      <c r="D167" s="7" t="n"/>
+    </row>
+    <row r="168">
+      <c r="D168" s="7" t="n"/>
+    </row>
+    <row r="169">
+      <c r="D169" s="7" t="n"/>
+    </row>
+    <row r="170">
+      <c r="D170" s="7" t="n"/>
+    </row>
+    <row r="171">
+      <c r="D171" s="7" t="n"/>
+    </row>
+    <row r="172">
+      <c r="D172" s="7" t="n"/>
+    </row>
+    <row r="173">
+      <c r="D173" s="7" t="n"/>
+    </row>
+    <row r="174">
+      <c r="D174" s="7" t="n"/>
+    </row>
+    <row r="175">
+      <c r="D175" s="7" t="n"/>
+    </row>
+    <row r="176">
+      <c r="D176" s="7" t="n"/>
+    </row>
+    <row r="177">
+      <c r="D177" s="7" t="n"/>
+    </row>
+    <row r="178">
+      <c r="D178" s="7" t="n"/>
+    </row>
+    <row r="179">
+      <c r="D179" s="7" t="n"/>
+    </row>
+    <row r="180">
+      <c r="D180" s="7" t="n"/>
+    </row>
+    <row r="181">
+      <c r="D181" s="7" t="n"/>
+    </row>
+    <row r="182">
+      <c r="D182" s="7" t="n"/>
+    </row>
+    <row r="183">
+      <c r="D183" s="7" t="n"/>
+    </row>
+    <row r="184">
+      <c r="D184" s="7" t="n"/>
+    </row>
+    <row r="185">
+      <c r="D185" s="7" t="n"/>
+    </row>
+    <row r="186">
+      <c r="D186" s="7" t="n"/>
+    </row>
+    <row r="187">
+      <c r="D187" s="7" t="n"/>
+    </row>
+    <row r="188">
+      <c r="D188" s="7" t="n"/>
+    </row>
+    <row r="189">
+      <c r="D189" s="7" t="n"/>
+    </row>
+    <row r="190">
+      <c r="D190" s="7" t="n"/>
+    </row>
+    <row r="191">
+      <c r="D191" s="7" t="n"/>
+    </row>
+    <row r="192">
+      <c r="D192" s="7" t="n"/>
+    </row>
+    <row r="193">
+      <c r="D193" s="7" t="n"/>
+    </row>
+    <row r="194">
+      <c r="D194" s="7" t="n"/>
+    </row>
+    <row r="195">
+      <c r="D195" s="7" t="n"/>
+    </row>
+    <row r="196">
+      <c r="D196" s="7" t="n"/>
+    </row>
+    <row r="197">
+      <c r="D197" s="7" t="n"/>
+    </row>
+    <row r="198">
+      <c r="D198" s="7" t="n"/>
+    </row>
+    <row r="199">
+      <c r="D199" s="7" t="n"/>
+    </row>
+    <row r="200">
+      <c r="D200" s="7" t="n"/>
+    </row>
+    <row r="201">
+      <c r="D201" s="7" t="n"/>
+    </row>
+    <row r="202">
+      <c r="D202" s="7" t="n"/>
+    </row>
+    <row r="203">
+      <c r="D203" s="7" t="n"/>
+    </row>
+    <row r="204">
+      <c r="D204" s="7" t="n"/>
+    </row>
+    <row r="205">
+      <c r="D205" s="7" t="n"/>
+    </row>
+    <row r="206">
+      <c r="D206" s="7" t="n"/>
+    </row>
+    <row r="207">
+      <c r="D207" s="7" t="n"/>
+    </row>
+    <row r="208">
+      <c r="D208" s="7" t="n"/>
+    </row>
+    <row r="209">
+      <c r="D209" s="7" t="n"/>
+    </row>
+    <row r="210">
+      <c r="D210" s="7" t="n"/>
+    </row>
+    <row r="211">
+      <c r="D211" s="7" t="n"/>
+    </row>
+    <row r="212">
+      <c r="D212" s="7" t="n"/>
+    </row>
+    <row r="213">
+      <c r="D213" s="7" t="n"/>
+    </row>
+    <row r="214">
+      <c r="D214" s="7" t="n"/>
+    </row>
+    <row r="215">
+      <c r="D215" s="7" t="n"/>
+    </row>
+    <row r="216">
+      <c r="D216" s="7" t="n"/>
+    </row>
+    <row r="217">
+      <c r="D217" s="7" t="n"/>
+    </row>
+    <row r="218">
+      <c r="D218" s="7" t="n"/>
+    </row>
+    <row r="219">
+      <c r="D219" s="7" t="n"/>
+    </row>
+    <row r="220">
+      <c r="D220" s="7" t="n"/>
+    </row>
+    <row r="221">
+      <c r="D221" s="7" t="n"/>
+    </row>
+    <row r="222">
+      <c r="D222" s="7" t="n"/>
+    </row>
+    <row r="223">
+      <c r="D223" s="7" t="n"/>
+    </row>
+    <row r="224">
+      <c r="D224" s="7" t="n"/>
+    </row>
+    <row r="225">
+      <c r="D225" s="7" t="n"/>
+    </row>
+    <row r="226">
+      <c r="D226" s="7" t="n"/>
+    </row>
+    <row r="227">
+      <c r="D227" s="7" t="n"/>
+    </row>
+    <row r="228">
+      <c r="D228" s="7" t="n"/>
+    </row>
+    <row r="229">
+      <c r="D229" s="7" t="n"/>
+    </row>
+    <row r="230">
+      <c r="D230" s="7" t="n"/>
+    </row>
+    <row r="231">
+      <c r="D231" s="7" t="n"/>
+    </row>
+    <row r="232">
+      <c r="D232" s="7" t="n"/>
+    </row>
+    <row r="233">
+      <c r="D233" s="7" t="n"/>
+    </row>
+    <row r="234">
+      <c r="D234" s="7" t="n"/>
+    </row>
+    <row r="235">
+      <c r="D235" s="7" t="n"/>
+    </row>
+    <row r="236">
+      <c r="D236" s="7" t="n"/>
+    </row>
+    <row r="237">
+      <c r="D237" s="7" t="n"/>
+    </row>
+    <row r="238">
+      <c r="D238" s="7" t="n"/>
+    </row>
+    <row r="239">
+      <c r="D239" s="7" t="n"/>
+    </row>
+    <row r="240">
+      <c r="D240" s="7" t="n"/>
+    </row>
+    <row r="241">
+      <c r="D241" s="7" t="n"/>
+    </row>
+    <row r="242">
+      <c r="D242" s="7" t="n"/>
+    </row>
+    <row r="243">
+      <c r="D243" s="7" t="n"/>
+    </row>
+    <row r="244">
+      <c r="D244" s="7" t="n"/>
+    </row>
+    <row r="245">
+      <c r="D245" s="7" t="n"/>
+    </row>
+    <row r="246">
+      <c r="D246" s="7" t="n"/>
+    </row>
+    <row r="247">
+      <c r="D247" s="7" t="n"/>
+    </row>
+    <row r="248">
+      <c r="D248" s="7" t="n"/>
+    </row>
+    <row r="249">
+      <c r="D249" s="7" t="n"/>
+    </row>
+    <row r="250">
+      <c r="D250" s="7" t="n"/>
+    </row>
+    <row r="251">
+      <c r="D251" s="7" t="n"/>
+    </row>
+    <row r="252">
+      <c r="D252" s="7" t="n"/>
+    </row>
+    <row r="253">
+      <c r="D253" s="7" t="n"/>
+    </row>
+    <row r="254">
+      <c r="D254" s="7" t="n"/>
+    </row>
+    <row r="255">
+      <c r="D255" s="7" t="n"/>
+    </row>
+    <row r="256">
+      <c r="D256" s="7" t="n"/>
+    </row>
+    <row r="257">
+      <c r="D257" s="7" t="n"/>
+    </row>
+    <row r="258">
+      <c r="D258" s="7" t="n"/>
+    </row>
+    <row r="259">
+      <c r="D259" s="7" t="n"/>
+    </row>
+    <row r="260">
+      <c r="D260" s="7" t="n"/>
+    </row>
+    <row r="261">
+      <c r="D261" s="7" t="n"/>
+    </row>
+    <row r="262">
+      <c r="D262" s="7" t="n"/>
+    </row>
+    <row r="263">
+      <c r="D263" s="7" t="n"/>
+    </row>
+    <row r="264">
+      <c r="D264" s="7" t="n"/>
+    </row>
+    <row r="265">
+      <c r="D265" s="7" t="n"/>
+    </row>
+    <row r="266">
+      <c r="D266" s="7" t="n"/>
+    </row>
+    <row r="267">
+      <c r="D267" s="7" t="n"/>
+    </row>
+    <row r="268">
+      <c r="D268" s="7" t="n"/>
+    </row>
+    <row r="269">
+      <c r="D269" s="7" t="n"/>
+    </row>
+    <row r="270">
+      <c r="D270" s="7" t="n"/>
+    </row>
+    <row r="271">
+      <c r="D271" s="7" t="n"/>
+    </row>
+    <row r="272">
+      <c r="D272" s="7" t="n"/>
+    </row>
+    <row r="273">
+      <c r="D273" s="7" t="n"/>
+    </row>
+    <row r="274">
+      <c r="D274" s="7" t="n"/>
+    </row>
+    <row r="275">
+      <c r="D275" s="7" t="n"/>
+    </row>
+    <row r="276">
+      <c r="D276" s="7" t="n"/>
+    </row>
+    <row r="277">
+      <c r="D277" s="7" t="n"/>
+    </row>
+    <row r="278">
+      <c r="D278" s="7" t="n"/>
+    </row>
+    <row r="279">
+      <c r="D279" s="7" t="n"/>
+    </row>
+    <row r="280">
+      <c r="D280" s="7" t="n"/>
+    </row>
+    <row r="281">
+      <c r="D281" s="7" t="n"/>
+    </row>
+    <row r="282">
+      <c r="D282" s="7" t="n"/>
+    </row>
+    <row r="283">
+      <c r="D283" s="7" t="n"/>
+    </row>
+    <row r="284">
+      <c r="D284" s="7" t="n"/>
+    </row>
+    <row r="285">
+      <c r="D285" s="7" t="n"/>
+    </row>
+    <row r="286">
+      <c r="D286" s="7" t="n"/>
+    </row>
+    <row r="287">
+      <c r="D287" s="7" t="n"/>
+    </row>
+    <row r="288">
+      <c r="D288" s="7" t="n"/>
+    </row>
+    <row r="289">
+      <c r="D289" s="7" t="n"/>
+    </row>
+    <row r="290">
+      <c r="D290" s="7" t="n"/>
+    </row>
+    <row r="291">
+      <c r="D291" s="7" t="n"/>
+    </row>
+    <row r="292">
+      <c r="D292" s="7" t="n"/>
+    </row>
+    <row r="293">
+      <c r="D293" s="7" t="n"/>
+    </row>
+    <row r="294">
+      <c r="D294" s="7" t="n"/>
+    </row>
+    <row r="295">
+      <c r="D295" s="7" t="n"/>
+    </row>
+    <row r="296">
+      <c r="D296" s="7" t="n"/>
+    </row>
+    <row r="297">
+      <c r="D297" s="7" t="n"/>
+    </row>
+    <row r="298">
+      <c r="D298" s="7" t="n"/>
+    </row>
+    <row r="299">
+      <c r="D299" s="7" t="n"/>
+    </row>
+    <row r="300">
+      <c r="D300" s="7" t="n"/>
+    </row>
+    <row r="301">
+      <c r="D301" s="7" t="n"/>
+    </row>
+    <row r="302">
+      <c r="D302" s="7" t="n"/>
+    </row>
+    <row r="303">
+      <c r="D303" s="7" t="n"/>
+    </row>
+    <row r="304">
+      <c r="D304" s="7" t="n"/>
+    </row>
+    <row r="305">
+      <c r="D305" s="7" t="n"/>
+    </row>
+    <row r="306">
+      <c r="D306" s="7" t="n"/>
+    </row>
+    <row r="307">
+      <c r="D307" s="7" t="n"/>
+    </row>
+    <row r="308">
+      <c r="D308" s="7" t="n"/>
+    </row>
+    <row r="309">
+      <c r="D309" s="7" t="n"/>
+    </row>
+    <row r="310">
+      <c r="D310" s="7" t="n"/>
+    </row>
+    <row r="311">
+      <c r="D311" s="7" t="n"/>
+    </row>
+    <row r="312">
+      <c r="D312" s="7" t="n"/>
+    </row>
+    <row r="313">
+      <c r="D313" s="7" t="n"/>
+    </row>
+    <row r="314">
+      <c r="D314" s="7" t="n"/>
+    </row>
+    <row r="315">
+      <c r="D315" s="7" t="n"/>
+    </row>
+    <row r="316">
+      <c r="D316" s="7" t="n"/>
+    </row>
+    <row r="317">
+      <c r="D317" s="7" t="n"/>
+    </row>
+    <row r="318">
+      <c r="D318" s="7" t="n"/>
+    </row>
+    <row r="319">
+      <c r="D319" s="7" t="n"/>
+    </row>
+    <row r="320">
+      <c r="D320" s="7" t="n"/>
+    </row>
+    <row r="321">
+      <c r="D321" s="7" t="n"/>
+    </row>
+    <row r="322">
+      <c r="D322" s="7" t="n"/>
+    </row>
+    <row r="323">
+      <c r="D323" s="7" t="n"/>
+    </row>
+    <row r="324">
+      <c r="D324" s="7" t="n"/>
+    </row>
+    <row r="325">
+      <c r="D325" s="7" t="n"/>
+    </row>
+    <row r="326">
+      <c r="D326" s="7" t="n"/>
+    </row>
+    <row r="327">
+      <c r="D327" s="7" t="n"/>
+    </row>
+    <row r="328">
+      <c r="D328" s="7" t="n"/>
+    </row>
+    <row r="329">
+      <c r="D329" s="7" t="n"/>
+    </row>
+    <row r="330">
+      <c r="D330" s="7" t="n"/>
+    </row>
+    <row r="331">
+      <c r="D331" s="7" t="n"/>
+    </row>
+    <row r="332">
+      <c r="D332" s="7" t="n"/>
+    </row>
+    <row r="333">
+      <c r="D333" s="7" t="n"/>
+    </row>
+    <row r="334">
+      <c r="D334" s="7" t="n"/>
+    </row>
+    <row r="335">
+      <c r="D335" s="7" t="n"/>
+    </row>
+    <row r="336">
+      <c r="D336" s="7" t="n"/>
+    </row>
+    <row r="337">
+      <c r="D337" s="7" t="n"/>
+    </row>
+    <row r="338">
+      <c r="D338" s="7" t="n"/>
+    </row>
+    <row r="339">
+      <c r="D339" s="7" t="n"/>
+    </row>
+    <row r="340">
+      <c r="D340" s="7" t="n"/>
+    </row>
+    <row r="341">
+      <c r="D341" s="7" t="n"/>
+    </row>
+    <row r="342">
+      <c r="D342" s="7" t="n"/>
+    </row>
+    <row r="343">
+      <c r="D343" s="7" t="n"/>
+    </row>
+    <row r="344">
+      <c r="D344" s="7" t="n"/>
+    </row>
+    <row r="345">
+      <c r="D345" s="7" t="n"/>
+    </row>
+    <row r="346">
+      <c r="D346" s="7" t="n"/>
+    </row>
+    <row r="347">
+      <c r="D347" s="7" t="n"/>
+    </row>
+    <row r="348">
+      <c r="D348" s="7" t="n"/>
+    </row>
+    <row r="349">
+      <c r="D349" s="7" t="n"/>
+    </row>
+    <row r="350">
+      <c r="D350" s="7" t="n"/>
+    </row>
+    <row r="351">
+      <c r="D351" s="7" t="n"/>
+    </row>
+    <row r="352">
+      <c r="D352" s="7" t="n"/>
+    </row>
+    <row r="353">
+      <c r="D353" s="7" t="n"/>
+    </row>
+    <row r="354">
+      <c r="D354" s="7" t="n"/>
+    </row>
+    <row r="355">
+      <c r="D355" s="7" t="n"/>
+    </row>
+    <row r="356">
+      <c r="D356" s="7" t="n"/>
+    </row>
+    <row r="357">
+      <c r="D357" s="7" t="n"/>
+    </row>
+    <row r="358">
+      <c r="D358" s="7" t="n"/>
+    </row>
+    <row r="359">
+      <c r="D359" s="7" t="n"/>
+    </row>
+    <row r="360">
+      <c r="D360" s="7" t="n"/>
+    </row>
+    <row r="361">
+      <c r="D361" s="7" t="n"/>
+    </row>
+    <row r="362">
+      <c r="D362" s="7" t="n"/>
+    </row>
+    <row r="363">
+      <c r="D363" s="7" t="n"/>
+    </row>
+    <row r="364">
+      <c r="D364" s="7" t="n"/>
+    </row>
+    <row r="365">
+      <c r="D365" s="7" t="n"/>
+    </row>
+    <row r="366">
+      <c r="D366" s="7" t="n"/>
+    </row>
+    <row r="367">
+      <c r="D367" s="7" t="n"/>
+    </row>
+    <row r="368">
+      <c r="D368" s="7" t="n"/>
+    </row>
+    <row r="369">
+      <c r="D369" s="7" t="n"/>
+    </row>
+    <row r="370">
+      <c r="D370" s="7" t="n"/>
+    </row>
+    <row r="371">
+      <c r="D371" s="7" t="n"/>
+    </row>
+    <row r="372">
+      <c r="D372" s="7" t="n"/>
+    </row>
+    <row r="373">
+      <c r="D373" s="7" t="n"/>
+    </row>
+    <row r="374">
+      <c r="D374" s="7" t="n"/>
+    </row>
+    <row r="375">
+      <c r="D375" s="7" t="n"/>
+    </row>
+    <row r="376">
+      <c r="D376" s="7" t="n"/>
+    </row>
+    <row r="377">
+      <c r="D377" s="7" t="n"/>
+    </row>
+    <row r="378">
+      <c r="D378" s="7" t="n"/>
+    </row>
+    <row r="379">
+      <c r="D379" s="7" t="n"/>
+    </row>
+    <row r="380">
+      <c r="D380" s="7" t="n"/>
+    </row>
+    <row r="381">
+      <c r="D381" s="7" t="n"/>
+    </row>
+    <row r="382">
+      <c r="D382" s="7" t="n"/>
+    </row>
+    <row r="383">
+      <c r="D383" s="7" t="n"/>
+    </row>
+    <row r="384">
+      <c r="D384" s="7" t="n"/>
+    </row>
+    <row r="385">
+      <c r="D385" s="7" t="n"/>
+    </row>
+    <row r="386">
+      <c r="D386" s="7" t="n"/>
+    </row>
+    <row r="387">
+      <c r="D387" s="7" t="n"/>
+    </row>
+    <row r="388">
+      <c r="D388" s="7" t="n"/>
+    </row>
+    <row r="389">
+      <c r="D389" s="7" t="n"/>
+    </row>
+    <row r="390">
+      <c r="D390" s="7" t="n"/>
+    </row>
+    <row r="391">
+      <c r="D391" s="7" t="n"/>
+    </row>
+    <row r="392">
+      <c r="D392" s="7" t="n"/>
+    </row>
+    <row r="393">
+      <c r="D393" s="7" t="n"/>
+    </row>
+    <row r="394">
+      <c r="D394" s="7" t="n"/>
+    </row>
+    <row r="395">
+      <c r="D395" s="7" t="n"/>
+    </row>
+    <row r="396">
+      <c r="D396" s="7" t="n"/>
+    </row>
+    <row r="397">
+      <c r="D397" s="7" t="n"/>
+    </row>
+    <row r="398">
+      <c r="D398" s="7" t="n"/>
+    </row>
+    <row r="399">
+      <c r="D399" s="7" t="n"/>
+    </row>
+    <row r="400">
+      <c r="D400" s="7" t="n"/>
+    </row>
+    <row r="401">
+      <c r="D401" s="7" t="n"/>
+    </row>
+    <row r="402">
+      <c r="D402" s="7" t="n"/>
+    </row>
+    <row r="403">
+      <c r="D403" s="7" t="n"/>
+    </row>
+    <row r="404">
+      <c r="D404" s="7" t="n"/>
+    </row>
+    <row r="405">
+      <c r="D405" s="7" t="n"/>
+    </row>
+    <row r="406">
+      <c r="D406" s="7" t="n"/>
+    </row>
+    <row r="407">
+      <c r="D407" s="7" t="n"/>
+    </row>
+    <row r="408">
+      <c r="D408" s="7" t="n"/>
+    </row>
+    <row r="409">
+      <c r="D409" s="7" t="n"/>
+    </row>
+    <row r="410">
+      <c r="D410" s="7" t="n"/>
+    </row>
+    <row r="411">
+      <c r="D411" s="7" t="n"/>
+    </row>
+    <row r="412">
+      <c r="D412" s="7" t="n"/>
+    </row>
+    <row r="413">
+      <c r="D413" s="7" t="n"/>
+    </row>
+    <row r="414">
+      <c r="D414" s="7" t="n"/>
+    </row>
+    <row r="415">
+      <c r="D415" s="7" t="n"/>
+    </row>
+    <row r="416">
+      <c r="D416" s="7" t="n"/>
+    </row>
+    <row r="417">
+      <c r="D417" s="7" t="n"/>
+    </row>
+    <row r="418">
+      <c r="D418" s="7" t="n"/>
+    </row>
+    <row r="419">
+      <c r="D419" s="7" t="n"/>
+    </row>
+    <row r="420">
+      <c r="D420" s="7" t="n"/>
+    </row>
+    <row r="421">
+      <c r="D421" s="7" t="n"/>
+    </row>
+    <row r="422">
+      <c r="D422" s="7" t="n"/>
+    </row>
+    <row r="423">
+      <c r="D423" s="7" t="n"/>
+    </row>
+    <row r="424">
+      <c r="D424" s="7" t="n"/>
+    </row>
+    <row r="425">
+      <c r="D425" s="7" t="n"/>
+    </row>
+    <row r="426">
+      <c r="D426" s="7" t="n"/>
+    </row>
+    <row r="427">
+      <c r="D427" s="7" t="n"/>
+    </row>
+    <row r="428">
+      <c r="D428" s="7" t="n"/>
+    </row>
+    <row r="429">
+      <c r="D429" s="7" t="n"/>
+    </row>
+    <row r="430">
+      <c r="D430" s="7" t="n"/>
+    </row>
+    <row r="431">
+      <c r="D431" s="7" t="n"/>
+    </row>
+    <row r="432">
+      <c r="D432" s="7" t="n"/>
+    </row>
+    <row r="433">
+      <c r="D433" s="7" t="n"/>
+    </row>
+    <row r="434">
+      <c r="D434" s="7" t="n"/>
+    </row>
+    <row r="435">
+      <c r="D435" s="7" t="n"/>
+    </row>
+    <row r="436">
+      <c r="D436" s="7" t="n"/>
+    </row>
+    <row r="437">
+      <c r="D437" s="7" t="n"/>
+    </row>
+    <row r="438">
+      <c r="D438" s="7" t="n"/>
+    </row>
+    <row r="439">
+      <c r="D439" s="7" t="n"/>
+    </row>
+    <row r="440">
+      <c r="D440" s="7" t="n"/>
+    </row>
+    <row r="441">
+      <c r="D441" s="7" t="n"/>
+    </row>
+    <row r="442">
+      <c r="D442" s="7" t="n"/>
+    </row>
+    <row r="443">
+      <c r="D443" s="7" t="n"/>
+    </row>
+    <row r="444">
+      <c r="D444" s="7" t="n"/>
+    </row>
+    <row r="445">
+      <c r="D445" s="7" t="n"/>
+    </row>
+    <row r="446">
+      <c r="D446" s="7" t="n"/>
+    </row>
+    <row r="447">
+      <c r="D447" s="7" t="n"/>
+    </row>
+    <row r="448">
+      <c r="D448" s="7" t="n"/>
+    </row>
+    <row r="449">
+      <c r="D449" s="7" t="n"/>
+    </row>
+    <row r="450">
+      <c r="D450" s="7" t="n"/>
+    </row>
+    <row r="451">
+      <c r="D451" s="7" t="n"/>
+    </row>
+    <row r="452">
+      <c r="D452" s="7" t="n"/>
+    </row>
+    <row r="453">
+      <c r="D453" s="7" t="n"/>
+    </row>
+    <row r="454">
+      <c r="D454" s="7" t="n"/>
+    </row>
+    <row r="455">
+      <c r="D455" s="7" t="n"/>
+    </row>
+    <row r="456">
+      <c r="D456" s="7" t="n"/>
+    </row>
+    <row r="457">
+      <c r="D457" s="7" t="n"/>
+    </row>
+    <row r="458">
+      <c r="D458" s="7" t="n"/>
+    </row>
+    <row r="459">
+      <c r="D459" s="7" t="n"/>
+    </row>
+    <row r="460">
+      <c r="D460" s="7" t="n"/>
+    </row>
+    <row r="461">
+      <c r="D461" s="7" t="n"/>
+    </row>
+    <row r="462">
+      <c r="D462" s="7" t="n"/>
+    </row>
+    <row r="463">
+      <c r="D463" s="7" t="n"/>
+    </row>
+    <row r="464">
+      <c r="D464" s="7" t="n"/>
+    </row>
+    <row r="465">
+      <c r="D465" s="7" t="n"/>
+    </row>
+    <row r="466">
+      <c r="D466" s="7" t="n"/>
+    </row>
+    <row r="467">
+      <c r="D467" s="7" t="n"/>
+    </row>
+    <row r="468">
+      <c r="D468" s="7" t="n"/>
+    </row>
+    <row r="469">
+      <c r="D469" s="7" t="n"/>
+    </row>
+    <row r="470">
+      <c r="D470" s="7" t="n"/>
+    </row>
+    <row r="471">
+      <c r="D471" s="7" t="n"/>
+    </row>
+    <row r="472">
+      <c r="D472" s="7" t="n"/>
+    </row>
+    <row r="473">
+      <c r="D473" s="7" t="n"/>
+    </row>
+    <row r="474">
+      <c r="D474" s="7" t="n"/>
+    </row>
+    <row r="475">
+      <c r="D475" s="7" t="n"/>
+    </row>
+    <row r="476">
+      <c r="D476" s="7" t="n"/>
+    </row>
+    <row r="477">
+      <c r="D477" s="7" t="n"/>
+    </row>
+    <row r="478">
+      <c r="D478" s="7" t="n"/>
+    </row>
+    <row r="479">
+      <c r="D479" s="7" t="n"/>
+    </row>
+    <row r="480">
+      <c r="D480" s="7" t="n"/>
+    </row>
+    <row r="481">
+      <c r="D481" s="7" t="n"/>
+    </row>
+    <row r="482">
+      <c r="D482" s="7" t="n"/>
+    </row>
+    <row r="483">
+      <c r="D483" s="7" t="n"/>
+    </row>
+    <row r="484">
+      <c r="D484" s="7" t="n"/>
+    </row>
+    <row r="485">
+      <c r="D485" s="7" t="n"/>
+    </row>
+    <row r="486">
+      <c r="D486" s="7" t="n"/>
+    </row>
+    <row r="487">
+      <c r="D487" s="7" t="n"/>
+    </row>
+    <row r="488">
+      <c r="D488" s="7" t="n"/>
+    </row>
+    <row r="489">
+      <c r="D489" s="7" t="n"/>
+    </row>
+    <row r="490">
+      <c r="D490" s="7" t="n"/>
+    </row>
+    <row r="491">
+      <c r="D491" s="7" t="n"/>
+    </row>
+    <row r="492">
+      <c r="D492" s="7" t="n"/>
+    </row>
+    <row r="493">
+      <c r="D493" s="7" t="n"/>
+    </row>
+    <row r="494">
+      <c r="D494" s="7" t="n"/>
+    </row>
+    <row r="495">
+      <c r="D495" s="7" t="n"/>
+    </row>
+    <row r="496">
+      <c r="D496" s="7" t="n"/>
+    </row>
+    <row r="497">
+      <c r="D497" s="7" t="n"/>
+    </row>
+    <row r="498">
+      <c r="D498" s="7" t="n"/>
+    </row>
+    <row r="499">
+      <c r="D499" s="7" t="n"/>
+    </row>
+    <row r="500">
+      <c r="D500" s="7" t="n"/>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>SA2</t>
+        </is>
+      </c>
+      <c r="D501" s="9" t="n">
+        <v>46346</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>